<commit_message>
Add README and Glossary tabs to all exercise and template Excel files
Every Excel file (10 files) now has:

README tab (first sheet):
- Explains what the exercise/template is for
- How to use the file (yellow cells = your input, white = formulas)
- What you are calculating, with plain-language formulas
- Account-type-specific instructions (extent, condition, services, OESA, OTSA)

Glossary tab:
- 22 terms defined: GVA, GDP, IC, Output, SUT, SNA, SEEA-EA, OESA,
  OTSA, Partial, CI, NCP, SCC, Mg CO2, ha, kg/yr, USD million, ISIC,
  SIC, EEZ, RAG, and more
- Each term has: abbreviation, full name, plain definition, and unit

Also fixed abbreviated units throughout all sheets:
- "(M)" replaced with "(USD million)" for clarity
- All technical terms now have their full names on first use

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s-s-event-bogor/sessions/day-2/clinic/condition/condition_account_template.xlsx
+++ b/s-s-event-bogor/sessions/day-2/clinic/condition/condition_account_template.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condition Account" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Levels" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condition Account" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Levels" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +56,12 @@
       <name val="Arial"/>
       <color rgb="003B9C7B"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000A5455"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -102,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,6 +128,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,6 +497,73 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="000A5455"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ocean Accounting Clinic: Condition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Account Template</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>How to use this file</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Fill in the yellow cells with your country's data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>White cells with formulas will calculate automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>See the Glossary sheet for definitions of all terms and abbreviations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>See the Instructions sheet (if present) for detailed step-by-step guidance.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="003B9C7B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -539,6 +620,7 @@
       </c>
       <c r="D4" s="3" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -794,7 +876,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="000A5455"/>
@@ -829,6 +911,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1431,7 +1514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1533,4 +1616,502 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="003B9C7B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Glossary of Terms and Abbreviations</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Term / Abbreviation</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Full Name</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>GVA</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Gross Value Added</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Total output minus intermediate consumption. The value an industry adds to the economy.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Currency (e.g., USD, local currency)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>GDP</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Gross Domestic Product</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Total value of goods and services produced in a country. Sum of GVA across all industries plus taxes minus subsidies.</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>IC</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Intermediate Consumption</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>The value of goods and services consumed as inputs during production (e.g., fuel, raw materials, purchased services). Does not include fixed assets.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Gross Output</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Total value of goods and services produced by an industry before deducting input costs. Also called gross sales or turnover.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>SUT</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Supply-Use Tables</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Statistical tables from the national accounts showing what each industry produces (supply) and what each industry consumes (use). Published by the National Statistical Office.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>SNA</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>System of National Accounts</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>The international statistical standard for measuring economic activity. Published by the UN. The basis for GDP calculation.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>SEEA-EA</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>System of Environmental-Economic Accounting - Ecosystem Accounting</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>The international statistical standard for measuring ecosystems, their condition, and the services they provide.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>OESA</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Ocean Economy Satellite Account</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>A satellite account that reorganizes national accounts to identify the market-based ocean economy. Reports GDP-compatible indicators.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>OTSA</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Ocean Tourism Satellite Account</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>A satellite account focused on coastal and marine tourism's economic contribution. A subset of OESA.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Ocean Economy Partial</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>The share (0 to 1) of a mixed industry's output that is ocean-related. For example, if 30% of construction is coastal, the partial is 0.30.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Proportion (0 to 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Condition Index</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>A normalized score from 0 (fully degraded) to 1 (reference/healthy condition). Used in SEEA-EA condition accounts.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Index (0 to 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>NCP</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Net Carbon Production</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>The rate at which an ecosystem sequesters carbon dioxide per unit area per year.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Mg CO2/ha/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>SCC</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Social Cost of Carbon</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>An estimate of the economic damage caused by emitting one additional tonne of CO2. Used to value carbon sequestration.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>USD per Mg CO2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Mg CO2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Megagrams of CO2</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Metric tonnes of carbon dioxide. 1 Mg = 1 tonne = 1,000 kg.</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Mass</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>ha</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Hectares</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Unit of area. 1 hectare = 10,000 square metres = 0.01 square kilometres.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>kg/yr</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Kilograms per year</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Physical quantity measured in kilograms over one year.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Mass per time</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>USD million</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>United States Dollars, millions</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Monetary values expressed in millions of US dollars. For example, USD 132.5 million = USD 132,500,000.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>R million</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>South African Rand, millions</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Monetary values in the South Africa example are in millions of Rand.</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>ISIC</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>International Standard Industrial Classification</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>The UN classification system for economic activities. Used to map industries to ocean economy groups.</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>SIC</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Standard Industrial Classification</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>National classification system for economic activities. Varies by country but based on ISIC.</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>EEZ</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Exclusive Economic Zone</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>Maritime zone extending 200 nautical miles from a country's coastline, within which the country has rights to marine resources.</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Red-Amber-Green</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>A confidence rating system. Green = high confidence (direct evidence). Amber = moderate (proxy data). Red = low (sparse evidence).</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>